<commit_message>
Updated test and reporting
</commit_message>
<xml_diff>
--- a/ppt/tests.xlsx
+++ b/ppt/tests.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="141">
   <si>
     <t xml:space="preserve">TestCase ID</t>
   </si>
@@ -55,6 +55,9 @@
     <t xml:space="preserve">Homepage Renders successfully</t>
   </si>
   <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC_HOME_02</t>
   </si>
   <si>
@@ -71,6 +74,375 @@
   </si>
   <si>
     <t xml:space="preserve">TC_HOME_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login Option Visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check Navbar when logged out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login Button is visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_HOME_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign up option visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign up Button is visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_HOME_05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Featured vehicles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check Page for featured vehicles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Featured Vehicles should be visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_LOGIN_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User login with valid credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter correct email &amp; password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid email/password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login successful, modal closes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_LOGIN_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid login handling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter wrong password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid email + wrong password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error message shown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_LOGIN_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empty fields validation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submit empty form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empty fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validation error shown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_LOGIN_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modal close functionality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click close button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modal closes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_SIGNUP_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User signup with valid data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fill all fields correctly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account created successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_SIGNUP_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email validation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter invalid email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_SIGNUP_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Password validation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weak password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validation error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_SIGNUP_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required fields check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error messages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_SEARCH_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Search vehicles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter location/date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle list displayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_SEARCH_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No results case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Search unavailable vehicles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid criteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“No vehicles found” message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_SEARCH_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filter functionality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply filters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filter inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtered results shown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_SEARCH_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navigation to details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click vehicle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle click</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redirect to Vehicle Detail Page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_VEH_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Display vehicle details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open vehicle page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Details shown correctly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_VEH_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking option</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click “Book Now”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Button click</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking initiated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_VEH_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid vehicle ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open wrong ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error or fallback page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_BOOK_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">View bookings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open bookings page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logged-in user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking list displayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_BOOK_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No bookings case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No bookings exist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“No bookings” message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_BOOK_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click booking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking click</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking details shown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_PROF_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">View profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open profile page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User details displayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_PROF_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edit details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profile updated successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_PROF_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unauthorized access</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access without login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redirect to login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_ADMIN_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin access control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open admin page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-admin user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access denied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_ADMIN_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">View all bookings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All bookings displayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_ADMIN_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manage vehicles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add/Edit/Delete vehicle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changes reflected</t>
   </si>
 </sst>
 </file>
@@ -85,6 +457,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -106,6 +479,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -150,13 +524,25 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -282,77 +668,638 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="27.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="E3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>16</v>
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="11.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="16.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J10:K10"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>